<commit_message>
Added new content from stream.
</commit_message>
<xml_diff>
--- a/Logs/Incoming Inspection Logs/MDL-004_Incoming_Inspection.xlsx
+++ b/Logs/Incoming Inspection Logs/MDL-004_Incoming_Inspection.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="66">
   <si>
     <t xml:space="preserve">Incoming Inspection Log</t>
   </si>
@@ -79,6 +79,147 @@
   </si>
   <si>
     <t xml:space="preserve">CC0603226010AABX5R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P00002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mouser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC1206106050AAAX7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC0603104050AAAX7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC1210226025AAAX7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC0805226025AABX5R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CEA771MS107M1JLAS018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC0603103050AAAX7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC0603474050AAAX7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KPTBP04R1-500-02BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KPTBP04R1-500-03BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KPTBP04R1-500-04BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KUSB4105-GF-A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KHS4B-PH-SM4-TB(LF)(SN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DLQ62702P5179</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSSS26SHE3_B_H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TVSCDSOT23-SM712</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DLLS R976-NR-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMAP63203WU-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMAP63205WU-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP32-WROOM-32UE-N16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UCP2102C-A01-GQFN28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UDRV8825PWPR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTMP36GRTZ-REEL7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LSRP2512-2R2M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QTCMT1600T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QBC847BDW1T1G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0603330075AAA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0603510075AAA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0603682075AAA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC060310K2075AAA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805121150AAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC12101K2200AAC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC060322K1075AAA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC060347K5075AAA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC06031K0075AAA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC06031M0075AAA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC08050R2075AAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC060350K075AAA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC060330K075AAA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SW435151014845</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TP5010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KPTBP04P1-500-02BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KPTBP04P1-500-03BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KPPHR-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PTSPH-002T-P0.5L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FANDC5V4040mmPWMTACH</t>
   </si>
 </sst>
 </file>
@@ -321,6 +462,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -472,740 +614,1752 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="5"/>
+      <c r="A6" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>21</v>
+      </c>
       <c r="G6" s="5"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="5"/>
+      <c r="H6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J6" s="5"/>
-      <c r="K6" s="3"/>
+      <c r="K6" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
+      <c r="M6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="5"/>
+      <c r="A7" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="G7" s="5"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="5"/>
+      <c r="H7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J7" s="5"/>
-      <c r="K7" s="3"/>
+      <c r="K7" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
+      <c r="M7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="5"/>
+      <c r="A8" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="G8" s="5"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="5"/>
+      <c r="H8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J8" s="5"/>
-      <c r="K8" s="3"/>
+      <c r="K8" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
+      <c r="M8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="5"/>
+      <c r="A9" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="G9" s="5"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="5"/>
+      <c r="H9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J9" s="5"/>
-      <c r="K9" s="3"/>
+      <c r="K9" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
+      <c r="M9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="5"/>
+      <c r="A10" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="G10" s="5"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="5"/>
+      <c r="H10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J10" s="5"/>
-      <c r="K10" s="3"/>
+      <c r="K10" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
+      <c r="M10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N10" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="5"/>
+      <c r="A11" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="G11" s="5"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="5"/>
+      <c r="H11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J11" s="5"/>
-      <c r="K11" s="3"/>
+      <c r="K11" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
+      <c r="M11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="5"/>
+      <c r="A12" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="G12" s="5"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="5"/>
+      <c r="H12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J12" s="5"/>
-      <c r="K12" s="3"/>
+      <c r="K12" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
+      <c r="M12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="5"/>
+      <c r="A13" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="G13" s="5"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="5"/>
+      <c r="H13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J13" s="5"/>
-      <c r="K13" s="3"/>
+      <c r="K13" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
+      <c r="M13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N13" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="5"/>
+      <c r="A14" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="G14" s="5"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="5"/>
+      <c r="H14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J14" s="5"/>
-      <c r="K14" s="3"/>
+      <c r="K14" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
+      <c r="M14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="5"/>
+      <c r="A15" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>30</v>
+      </c>
       <c r="G15" s="5"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="5"/>
+      <c r="H15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J15" s="5"/>
-      <c r="K15" s="3"/>
+      <c r="K15" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
+      <c r="M15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="5"/>
+      <c r="A16" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>31</v>
+      </c>
       <c r="G16" s="5"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="5"/>
+      <c r="H16" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J16" s="5"/>
-      <c r="K16" s="3"/>
+      <c r="K16" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
+      <c r="M16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="5"/>
+      <c r="A17" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>32</v>
+      </c>
       <c r="G17" s="5"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="5"/>
+      <c r="H17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J17" s="5"/>
-      <c r="K17" s="3"/>
+      <c r="K17" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
+      <c r="M17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N17" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="5"/>
+      <c r="A18" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="G18" s="5"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="5"/>
+      <c r="H18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J18" s="5"/>
-      <c r="K18" s="3"/>
+      <c r="K18" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
+      <c r="M18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N18" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="5"/>
+      <c r="A19" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="G19" s="5"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="5"/>
+      <c r="H19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J19" s="5"/>
-      <c r="K19" s="3"/>
+      <c r="K19" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
+      <c r="M19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N19" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="5"/>
+      <c r="A20" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>35</v>
+      </c>
       <c r="G20" s="5"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="5"/>
+      <c r="H20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J20" s="5"/>
-      <c r="K20" s="3"/>
+      <c r="K20" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
-      <c r="N20" s="3"/>
+      <c r="M20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N20" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="5"/>
+      <c r="A21" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="G21" s="5"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="5"/>
+      <c r="H21" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J21" s="5"/>
-      <c r="K21" s="3"/>
+      <c r="K21" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
-      <c r="N21" s="3"/>
+      <c r="M21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N21" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="5"/>
+      <c r="A22" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>37</v>
+      </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="5"/>
+      <c r="H22" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J22" s="5"/>
-      <c r="K22" s="3"/>
+      <c r="K22" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
-      <c r="N22" s="3"/>
+      <c r="M22" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N22" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="5"/>
+      <c r="A23" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>38</v>
+      </c>
       <c r="G23" s="5"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="5"/>
+      <c r="H23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J23" s="5"/>
-      <c r="K23" s="3"/>
+      <c r="K23" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
+      <c r="M23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N23" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="5"/>
+      <c r="A24" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="G24" s="5"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="5"/>
+      <c r="H24" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J24" s="5"/>
-      <c r="K24" s="3"/>
+      <c r="K24" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L24" s="3"/>
-      <c r="M24" s="3"/>
-      <c r="N24" s="3"/>
+      <c r="M24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N24" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="5"/>
+      <c r="A25" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>40</v>
+      </c>
       <c r="G25" s="5"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="5"/>
+      <c r="H25" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J25" s="5"/>
-      <c r="K25" s="3"/>
+      <c r="K25" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L25" s="3"/>
-      <c r="M25" s="3"/>
-      <c r="N25" s="3"/>
+      <c r="M25" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N25" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="5"/>
+      <c r="A26" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>41</v>
+      </c>
       <c r="G26" s="5"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="5"/>
+      <c r="H26" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J26" s="5"/>
-      <c r="K26" s="3"/>
+      <c r="K26" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L26" s="3"/>
-      <c r="M26" s="3"/>
-      <c r="N26" s="3"/>
+      <c r="M26" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N26" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="5"/>
+      <c r="A27" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="G27" s="5"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="5"/>
+      <c r="H27" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J27" s="5"/>
-      <c r="K27" s="3"/>
+      <c r="K27" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L27" s="3"/>
-      <c r="M27" s="3"/>
-      <c r="N27" s="3"/>
+      <c r="M27" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N27" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="5"/>
+      <c r="A28" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>43</v>
+      </c>
       <c r="G28" s="5"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="5"/>
+      <c r="H28" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J28" s="5"/>
-      <c r="K28" s="3"/>
+      <c r="K28" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
+      <c r="M28" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N28" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="5"/>
+      <c r="A29" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G29" s="5"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="5"/>
+      <c r="H29" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J29" s="5"/>
-      <c r="K29" s="3"/>
+      <c r="K29" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L29" s="3"/>
-      <c r="M29" s="3"/>
-      <c r="N29" s="3"/>
+      <c r="M29" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N29" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="5"/>
+      <c r="A30" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="G30" s="5"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="5"/>
+      <c r="H30" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J30" s="5"/>
-      <c r="K30" s="3"/>
+      <c r="K30" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L30" s="3"/>
-      <c r="M30" s="3"/>
-      <c r="N30" s="3"/>
+      <c r="M30" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N30" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="5"/>
+      <c r="A31" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="G31" s="5"/>
-      <c r="H31" s="3"/>
-      <c r="I31" s="5"/>
+      <c r="H31" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J31" s="5"/>
-      <c r="K31" s="3"/>
+      <c r="K31" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L31" s="3"/>
-      <c r="M31" s="3"/>
-      <c r="N31" s="3"/>
+      <c r="M31" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N31" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="5"/>
+      <c r="A32" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>47</v>
+      </c>
       <c r="G32" s="5"/>
-      <c r="H32" s="3"/>
-      <c r="I32" s="5"/>
+      <c r="H32" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J32" s="5"/>
-      <c r="K32" s="3"/>
+      <c r="K32" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L32" s="3"/>
-      <c r="M32" s="3"/>
-      <c r="N32" s="3"/>
+      <c r="M32" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N32" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="5"/>
+      <c r="A33" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="G33" s="5"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="5"/>
+      <c r="H33" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J33" s="5"/>
-      <c r="K33" s="3"/>
+      <c r="K33" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
-      <c r="N33" s="3"/>
+      <c r="M33" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N33" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="5"/>
+      <c r="A34" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="G34" s="5"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="5"/>
+      <c r="H34" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J34" s="5"/>
-      <c r="K34" s="3"/>
+      <c r="K34" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
-      <c r="N34" s="3"/>
+      <c r="M34" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N34" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="5"/>
+      <c r="A35" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="G35" s="5"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="5"/>
+      <c r="H35" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J35" s="5"/>
-      <c r="K35" s="3"/>
+      <c r="K35" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L35" s="3"/>
-      <c r="M35" s="3"/>
-      <c r="N35" s="3"/>
+      <c r="M35" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N35" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="5"/>
+      <c r="A36" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>51</v>
+      </c>
       <c r="G36" s="5"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="5"/>
+      <c r="H36" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J36" s="5"/>
-      <c r="K36" s="3"/>
+      <c r="K36" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L36" s="3"/>
-      <c r="M36" s="3"/>
-      <c r="N36" s="3"/>
+      <c r="M36" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N36" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="5"/>
+      <c r="A37" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>52</v>
+      </c>
       <c r="G37" s="5"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="5"/>
+      <c r="H37" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J37" s="5"/>
-      <c r="K37" s="3"/>
+      <c r="K37" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L37" s="3"/>
-      <c r="M37" s="3"/>
-      <c r="N37" s="3"/>
+      <c r="M37" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N37" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
-      <c r="F38" s="5"/>
+      <c r="A38" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="G38" s="5"/>
-      <c r="H38" s="3"/>
-      <c r="I38" s="5"/>
+      <c r="H38" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J38" s="5"/>
-      <c r="K38" s="3"/>
+      <c r="K38" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L38" s="3"/>
-      <c r="M38" s="3"/>
-      <c r="N38" s="3"/>
+      <c r="M38" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N38" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
-      <c r="F39" s="5"/>
+      <c r="A39" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>54</v>
+      </c>
       <c r="G39" s="5"/>
-      <c r="H39" s="3"/>
-      <c r="I39" s="5"/>
+      <c r="H39" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I39" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J39" s="5"/>
-      <c r="K39" s="3"/>
+      <c r="K39" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
-      <c r="N39" s="3"/>
+      <c r="M39" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N39" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
-      <c r="F40" s="5"/>
+      <c r="A40" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="G40" s="5"/>
-      <c r="H40" s="3"/>
-      <c r="I40" s="5"/>
+      <c r="H40" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I40" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J40" s="5"/>
-      <c r="K40" s="3"/>
+      <c r="K40" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L40" s="3"/>
-      <c r="M40" s="3"/>
-      <c r="N40" s="3"/>
+      <c r="M40" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N40" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
-      <c r="F41" s="5"/>
+      <c r="A41" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>56</v>
+      </c>
       <c r="G41" s="5"/>
-      <c r="H41" s="3"/>
-      <c r="I41" s="5"/>
+      <c r="H41" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I41" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J41" s="5"/>
-      <c r="K41" s="3"/>
+      <c r="K41" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L41" s="3"/>
-      <c r="M41" s="3"/>
-      <c r="N41" s="3"/>
+      <c r="M41" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N41" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-      <c r="F42" s="5"/>
+      <c r="A42" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="G42" s="5"/>
-      <c r="H42" s="3"/>
-      <c r="I42" s="5"/>
+      <c r="H42" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I42" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J42" s="5"/>
-      <c r="K42" s="3"/>
+      <c r="K42" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L42" s="3"/>
-      <c r="M42" s="3"/>
-      <c r="N42" s="3"/>
+      <c r="M42" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N42" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
-      <c r="F43" s="5"/>
+      <c r="A43" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>58</v>
+      </c>
       <c r="G43" s="5"/>
-      <c r="H43" s="3"/>
-      <c r="I43" s="5"/>
+      <c r="H43" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I43" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J43" s="5"/>
-      <c r="K43" s="3"/>
+      <c r="K43" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L43" s="3"/>
-      <c r="M43" s="3"/>
-      <c r="N43" s="3"/>
+      <c r="M43" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N43" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
-      <c r="E44" s="3"/>
-      <c r="F44" s="5"/>
+      <c r="A44" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>59</v>
+      </c>
       <c r="G44" s="5"/>
-      <c r="H44" s="3"/>
-      <c r="I44" s="5"/>
+      <c r="H44" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I44" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J44" s="5"/>
-      <c r="K44" s="3"/>
+      <c r="K44" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L44" s="3"/>
-      <c r="M44" s="3"/>
-      <c r="N44" s="3"/>
+      <c r="M44" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N44" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-      <c r="F45" s="5"/>
+      <c r="A45" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>60</v>
+      </c>
       <c r="G45" s="5"/>
-      <c r="H45" s="3"/>
-      <c r="I45" s="5"/>
+      <c r="H45" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J45" s="5"/>
-      <c r="K45" s="3"/>
+      <c r="K45" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L45" s="3"/>
-      <c r="M45" s="3"/>
-      <c r="N45" s="3"/>
+      <c r="M45" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
-      <c r="F46" s="5"/>
+      <c r="A46" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>61</v>
+      </c>
       <c r="G46" s="5"/>
-      <c r="H46" s="3"/>
-      <c r="I46" s="5"/>
+      <c r="H46" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J46" s="5"/>
-      <c r="K46" s="3"/>
+      <c r="K46" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L46" s="3"/>
-      <c r="M46" s="3"/>
-      <c r="N46" s="3"/>
+      <c r="M46" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N46" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="5"/>
+      <c r="A47" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="G47" s="5"/>
-      <c r="H47" s="3"/>
-      <c r="I47" s="5"/>
+      <c r="H47" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I47" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J47" s="5"/>
-      <c r="K47" s="3"/>
+      <c r="K47" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L47" s="3"/>
-      <c r="M47" s="3"/>
-      <c r="N47" s="3"/>
+      <c r="M47" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N47" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-      <c r="F48" s="5"/>
+      <c r="A48" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>30</v>
+      </c>
       <c r="G48" s="5"/>
-      <c r="H48" s="3"/>
-      <c r="I48" s="5"/>
+      <c r="H48" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J48" s="5"/>
-      <c r="K48" s="3"/>
+      <c r="K48" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L48" s="3"/>
-      <c r="M48" s="3"/>
-      <c r="N48" s="3"/>
+      <c r="M48" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N48" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-      <c r="F49" s="5"/>
+      <c r="A49" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="G49" s="5"/>
-      <c r="H49" s="3"/>
-      <c r="I49" s="5"/>
+      <c r="H49" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J49" s="5"/>
-      <c r="K49" s="3"/>
+      <c r="K49" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L49" s="3"/>
-      <c r="M49" s="3"/>
-      <c r="N49" s="3"/>
+      <c r="M49" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N49" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-      <c r="F50" s="5"/>
+      <c r="A50" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="G50" s="5"/>
-      <c r="H50" s="3"/>
-      <c r="I50" s="5"/>
+      <c r="H50" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J50" s="5"/>
-      <c r="K50" s="3"/>
+      <c r="K50" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L50" s="3"/>
-      <c r="M50" s="3"/>
-      <c r="N50" s="3"/>
+      <c r="M50" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N50" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
-      <c r="F51" s="5"/>
+      <c r="A51" s="4" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="F51" s="5" t="s">
+        <v>65</v>
+      </c>
       <c r="G51" s="5"/>
-      <c r="H51" s="3"/>
-      <c r="I51" s="5"/>
+      <c r="H51" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I51" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J51" s="5"/>
-      <c r="K51" s="3"/>
+      <c r="K51" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="L51" s="3"/>
-      <c r="M51" s="3"/>
-      <c r="N51" s="3"/>
+      <c r="M51" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N51" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3"/>

</xml_diff>